<commit_message>
Updated GRC_grids model - 2025-09-09 00:01
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1464DD0-E1F7-4A04-96DC-277F97314058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{911546D3-477E-4196-8098-A908735F874F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6848,7 +6848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A358ECA-1BB9-4B58-9D6C-A0966DD58303}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A758940-2545-47F1-B237-73728EA8F4C7}">
   <dimension ref="B2:C948"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-21 00:21
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0D86FC6-FC81-4024-A75A-C046C083A40B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45C8983F-4AFA-470A-82AE-41A7F6059208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F609E2-EA15-43EF-804C-897D4C84FC0D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BBEDBED-A0DF-48D4-B176-038AF5D19DD5}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-22 23:33
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73DCB839-22E9-470B-BDDB-033FEAD9D804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DB3ED15-F0EB-4894-8952-6F480BA4ADAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3945F54-0459-430F-ADD7-3B31EA8F4265}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5412661A-AB81-4E5B-9472-022B6107C4EE}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids model - 2025-09-26 22:06
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E1C8664-86AD-4C0B-8520-DF68788BC34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8621FD8-08A2-4983-A858-A095778B096C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABDC66FE-D2EC-46B8-B7AD-F5ADD411C1D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A0BAAF-8981-4053-B82A-205920A3D9A5}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>